<commit_message>
Lab 11 Library: shelves in spaced rows of three, islands between the rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MSjWpMgByR7PswdtguveBk
</commit_message>
<xml_diff>
--- a/tools/world/lab11/lab11_layout.xlsx
+++ b/tools/world/lab11/lab11_layout.xlsx
@@ -21045,12 +21045,12 @@
       </c>
       <c r="BK34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BL34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM34" s="15" t="inlineStr">
@@ -21075,12 +21075,12 @@
       </c>
       <c r="BQ34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BR34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS34" s="15" t="inlineStr">
@@ -21105,12 +21105,12 @@
       </c>
       <c r="BW34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY34" s="15" t="inlineStr">
@@ -21135,12 +21135,12 @@
       </c>
       <c r="CC34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE34" s="15" t="inlineStr">
@@ -21165,12 +21165,12 @@
       </c>
       <c r="CI34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK34" s="15" t="inlineStr">
@@ -21195,7 +21195,7 @@
       </c>
       <c r="CO34" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP34" s="15" t="inlineStr">
@@ -21650,17 +21650,17 @@
       </c>
       <c r="BK35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BL35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BM35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BN35" s="15" t="inlineStr">
@@ -21675,17 +21675,17 @@
       </c>
       <c r="BP35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BQ35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BR35" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BS35" s="15" t="inlineStr">
@@ -21700,22 +21700,22 @@
       </c>
       <c r="BU35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BV35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BW35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BX35" s="15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY35" s="15" t="inlineStr">
@@ -21725,42 +21725,42 @@
       </c>
       <c r="BZ35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CA35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CB35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CC35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD35" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CF35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CG35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CH35" s="15" t="inlineStr">
@@ -21770,22 +21770,22 @@
       </c>
       <c r="CI35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CK35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CL35" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CM35" s="15" t="inlineStr">
@@ -21800,12 +21800,12 @@
       </c>
       <c r="CO35" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP35" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ35" s="15" t="inlineStr">
@@ -22260,22 +22260,22 @@
       </c>
       <c r="BL36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BN36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BO36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BP36" s="15" t="inlineStr">
@@ -22290,42 +22290,42 @@
       </c>
       <c r="BR36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BT36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BU36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BV36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BW36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BZ36" s="15" t="inlineStr">
@@ -22340,42 +22340,42 @@
       </c>
       <c r="CB36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CC36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CF36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CG36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CH36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CI36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ36" s="15" t="inlineStr">
@@ -22390,17 +22390,17 @@
       </c>
       <c r="CL36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CM36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CN36" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CO36" s="15" t="inlineStr">
@@ -22875,12 +22875,12 @@
       </c>
       <c r="BN37" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="BO37" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BP37" s="15" t="inlineStr">
@@ -22925,12 +22925,12 @@
       </c>
       <c r="BX37" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>m</t>
         </is>
       </c>
       <c r="BY37" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BZ37" s="15" t="inlineStr">
@@ -22975,12 +22975,12 @@
       </c>
       <c r="CH37" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="CI37" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CJ37" s="15" t="inlineStr">
@@ -23480,12 +23480,12 @@
       </c>
       <c r="BN38" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BO38" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BP38" s="15" t="inlineStr">
@@ -23530,12 +23530,12 @@
       </c>
       <c r="BX38" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BY38" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BZ38" s="15" t="inlineStr">
@@ -23580,12 +23580,12 @@
       </c>
       <c r="CH38" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CI38" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CJ38" s="15" t="inlineStr">
@@ -24675,12 +24675,12 @@
       </c>
       <c r="BK40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BL40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM40" s="15" t="inlineStr">
@@ -24705,12 +24705,12 @@
       </c>
       <c r="BQ40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BR40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS40" s="15" t="inlineStr">
@@ -24735,12 +24735,12 @@
       </c>
       <c r="BW40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY40" s="15" t="inlineStr">
@@ -24765,12 +24765,12 @@
       </c>
       <c r="CC40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE40" s="15" t="inlineStr">
@@ -24795,12 +24795,12 @@
       </c>
       <c r="CI40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK40" s="15" t="inlineStr">
@@ -24825,12 +24825,12 @@
       </c>
       <c r="CO40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP40" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ40" s="15" t="inlineStr">
@@ -25280,17 +25280,17 @@
       </c>
       <c r="BK41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BL41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>s</t>
         </is>
       </c>
       <c r="BM41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BN41" s="15" t="inlineStr">
@@ -25305,17 +25305,17 @@
       </c>
       <c r="BP41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BQ41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BR41" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BS41" s="15" t="inlineStr">
@@ -25330,22 +25330,22 @@
       </c>
       <c r="BU41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BV41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BW41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BX41" s="15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY41" s="15" t="inlineStr">
@@ -25355,42 +25355,42 @@
       </c>
       <c r="BZ41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CA41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CB41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CC41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD41" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CF41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CG41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CH41" s="15" t="inlineStr">
@@ -25400,22 +25400,22 @@
       </c>
       <c r="CI41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CK41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="CL41" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CM41" s="15" t="inlineStr">
@@ -25430,12 +25430,12 @@
       </c>
       <c r="CO41" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP41" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ41" s="15" t="inlineStr">
@@ -25890,27 +25890,27 @@
       </c>
       <c r="BL42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BN42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BO42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BP42" s="15" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BQ42" s="15" t="inlineStr">
@@ -25920,42 +25920,42 @@
       </c>
       <c r="BR42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BT42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BU42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BV42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BW42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BZ42" s="15" t="inlineStr">
@@ -25970,47 +25970,47 @@
       </c>
       <c r="CB42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CC42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CF42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CG42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CH42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CI42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ42" s="15" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK42" s="15" t="inlineStr">
@@ -26020,17 +26020,17 @@
       </c>
       <c r="CL42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CM42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CN42" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CO42" s="15" t="inlineStr">
@@ -26530,12 +26530,12 @@
       </c>
       <c r="BS43" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>m</t>
         </is>
       </c>
       <c r="BT43" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BU43" s="15" t="inlineStr">
@@ -26580,12 +26580,12 @@
       </c>
       <c r="CC43" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="CD43" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CE43" s="15" t="inlineStr">
@@ -27135,12 +27135,12 @@
       </c>
       <c r="BS44" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BT44" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BU44" s="15" t="inlineStr">
@@ -27185,12 +27185,12 @@
       </c>
       <c r="CC44" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CD44" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CE44" s="15" t="inlineStr">
@@ -28305,12 +28305,12 @@
       </c>
       <c r="BK46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BL46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM46" s="15" t="inlineStr">
@@ -28335,12 +28335,12 @@
       </c>
       <c r="BQ46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BR46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS46" s="15" t="inlineStr">
@@ -28365,12 +28365,12 @@
       </c>
       <c r="BW46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY46" s="15" t="inlineStr">
@@ -28395,12 +28395,12 @@
       </c>
       <c r="CC46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE46" s="15" t="inlineStr">
@@ -28425,12 +28425,12 @@
       </c>
       <c r="CI46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK46" s="15" t="inlineStr">
@@ -28455,12 +28455,12 @@
       </c>
       <c r="CO46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP46" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ46" s="15" t="inlineStr">
@@ -28910,17 +28910,17 @@
       </c>
       <c r="BK47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BL47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BM47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BN47" s="15" t="inlineStr">
@@ -28935,17 +28935,17 @@
       </c>
       <c r="BP47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BQ47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BR47" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BS47" s="15" t="inlineStr">
@@ -28960,22 +28960,22 @@
       </c>
       <c r="BU47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BV47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>s</t>
         </is>
       </c>
       <c r="BW47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BX47" s="15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY47" s="15" t="inlineStr">
@@ -28985,42 +28985,42 @@
       </c>
       <c r="BZ47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CA47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CB47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CC47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD47" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CF47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CG47" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CH47" s="15" t="inlineStr">
@@ -29030,12 +29030,12 @@
       </c>
       <c r="CI47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK47" s="15" t="inlineStr">
@@ -29060,12 +29060,12 @@
       </c>
       <c r="CO47" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP47" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ47" s="15" t="inlineStr">
@@ -29520,22 +29520,22 @@
       </c>
       <c r="BL48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BN48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BO48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BP48" s="15" t="inlineStr">
@@ -29550,47 +29550,47 @@
       </c>
       <c r="BR48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BT48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BU48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BV48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BW48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BZ48" s="15" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CA48" s="15" t="inlineStr">
@@ -29600,42 +29600,42 @@
       </c>
       <c r="CB48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CC48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CF48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CG48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CH48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CI48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ48" s="15" t="inlineStr">
@@ -29650,17 +29650,17 @@
       </c>
       <c r="CL48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CM48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CN48" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CO48" s="15" t="inlineStr">
@@ -30135,12 +30135,12 @@
       </c>
       <c r="BN49" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>m</t>
         </is>
       </c>
       <c r="BO49" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BP49" s="15" t="inlineStr">
@@ -30185,12 +30185,12 @@
       </c>
       <c r="BX49" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="BY49" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BZ49" s="15" t="inlineStr">
@@ -30235,12 +30235,12 @@
       </c>
       <c r="CH49" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>m</t>
         </is>
       </c>
       <c r="CI49" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CJ49" s="15" t="inlineStr">
@@ -30740,12 +30740,12 @@
       </c>
       <c r="BN50" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BO50" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BP50" s="15" t="inlineStr">
@@ -30790,12 +30790,12 @@
       </c>
       <c r="BX50" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BY50" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BZ50" s="15" t="inlineStr">
@@ -30840,12 +30840,12 @@
       </c>
       <c r="CH50" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CI50" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CJ50" s="15" t="inlineStr">
@@ -31935,12 +31935,12 @@
       </c>
       <c r="BK52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BL52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM52" s="15" t="inlineStr">
@@ -31965,12 +31965,12 @@
       </c>
       <c r="BQ52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BR52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS52" s="15" t="inlineStr">
@@ -31995,12 +31995,12 @@
       </c>
       <c r="BW52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY52" s="15" t="inlineStr">
@@ -32025,12 +32025,12 @@
       </c>
       <c r="CC52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE52" s="15" t="inlineStr">
@@ -32055,12 +32055,12 @@
       </c>
       <c r="CI52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ52" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK52" s="15" t="inlineStr">
@@ -32540,17 +32540,17 @@
       </c>
       <c r="BK53" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BL53" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BM53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BN53" s="15" t="inlineStr">
@@ -32565,17 +32565,17 @@
       </c>
       <c r="BP53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BQ53" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BR53" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BS53" s="15" t="inlineStr">
@@ -32590,22 +32590,22 @@
       </c>
       <c r="BU53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BV53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BW53" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BX53" s="15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY53" s="15" t="inlineStr">
@@ -32615,42 +32615,42 @@
       </c>
       <c r="BZ53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CA53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CB53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CC53" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD53" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CF53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>s</t>
         </is>
       </c>
       <c r="CG53" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CH53" s="15" t="inlineStr">
@@ -32660,12 +32660,12 @@
       </c>
       <c r="CI53" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ53" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK53" s="15" t="inlineStr">
@@ -33150,22 +33150,22 @@
       </c>
       <c r="BL54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BN54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BO54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BP54" s="15" t="inlineStr">
@@ -33180,42 +33180,42 @@
       </c>
       <c r="BR54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BT54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BU54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BV54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BW54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BZ54" s="15" t="inlineStr">
@@ -33230,47 +33230,47 @@
       </c>
       <c r="CB54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CC54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CF54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CG54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CH54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CI54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ54" s="15" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK54" s="15" t="inlineStr">
@@ -33280,7 +33280,7 @@
       </c>
       <c r="CL54" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CM54" s="15" t="inlineStr">
@@ -33790,12 +33790,12 @@
       </c>
       <c r="BS55" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="BT55" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BU55" s="15" t="inlineStr">
@@ -33840,12 +33840,12 @@
       </c>
       <c r="CC55" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>m</t>
         </is>
       </c>
       <c r="CD55" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CE55" s="15" t="inlineStr">
@@ -34395,12 +34395,12 @@
       </c>
       <c r="BS56" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BT56" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BU56" s="15" t="inlineStr">
@@ -34445,12 +34445,12 @@
       </c>
       <c r="CC56" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CD56" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CE56" s="15" t="inlineStr">
@@ -35565,12 +35565,12 @@
       </c>
       <c r="BK58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BL58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM58" s="15" t="inlineStr">
@@ -35595,12 +35595,12 @@
       </c>
       <c r="BQ58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BR58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS58" s="15" t="inlineStr">
@@ -35625,12 +35625,12 @@
       </c>
       <c r="BW58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY58" s="15" t="inlineStr">
@@ -35655,12 +35655,12 @@
       </c>
       <c r="CC58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE58" s="15" t="inlineStr">
@@ -35685,12 +35685,12 @@
       </c>
       <c r="CI58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK58" s="15" t="inlineStr">
@@ -35715,12 +35715,12 @@
       </c>
       <c r="CO58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP58" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ58" s="15" t="inlineStr">
@@ -36170,17 +36170,17 @@
       </c>
       <c r="BK59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BL59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BM59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BN59" s="15" t="inlineStr">
@@ -36195,17 +36195,17 @@
       </c>
       <c r="BP59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BQ59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>s</t>
         </is>
       </c>
       <c r="BR59" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BS59" s="15" t="inlineStr">
@@ -36220,22 +36220,22 @@
       </c>
       <c r="BU59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BV59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BW59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BX59" s="15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY59" s="15" t="inlineStr">
@@ -36245,42 +36245,42 @@
       </c>
       <c r="BZ59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CA59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CB59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CC59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD59" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CF59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CG59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CH59" s="15" t="inlineStr">
@@ -36290,22 +36290,22 @@
       </c>
       <c r="CI59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CK59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CL59" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CM59" s="15" t="inlineStr">
@@ -36320,12 +36320,12 @@
       </c>
       <c r="CO59" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP59" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ59" s="15" t="inlineStr">
@@ -36780,27 +36780,27 @@
       </c>
       <c r="BL60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BN60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BO60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BP60" s="15" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BQ60" s="15" t="inlineStr">
@@ -36810,42 +36810,42 @@
       </c>
       <c r="BR60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BT60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BU60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BV60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BW60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BZ60" s="15" t="inlineStr">
@@ -36860,42 +36860,42 @@
       </c>
       <c r="CB60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CC60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CF60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CG60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CH60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CI60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ60" s="15" t="inlineStr">
@@ -36910,17 +36910,17 @@
       </c>
       <c r="CL60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CM60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CN60" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CO60" s="15" t="inlineStr">
@@ -37395,12 +37395,12 @@
       </c>
       <c r="BN61" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="BO61" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BP61" s="15" t="inlineStr">
@@ -37445,12 +37445,12 @@
       </c>
       <c r="BX61" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>m</t>
         </is>
       </c>
       <c r="BY61" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BZ61" s="15" t="inlineStr">
@@ -37495,12 +37495,12 @@
       </c>
       <c r="CH61" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="CI61" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CJ61" s="15" t="inlineStr">
@@ -38000,12 +38000,12 @@
       </c>
       <c r="BN62" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BO62" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BP62" s="15" t="inlineStr">
@@ -38050,12 +38050,12 @@
       </c>
       <c r="BX62" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BY62" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BZ62" s="15" t="inlineStr">
@@ -38100,12 +38100,12 @@
       </c>
       <c r="CH62" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CI62" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CJ62" s="15" t="inlineStr">
@@ -39195,12 +39195,12 @@
       </c>
       <c r="BK64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BL64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM64" s="15" t="inlineStr">
@@ -39225,12 +39225,12 @@
       </c>
       <c r="BQ64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BR64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS64" s="15" t="inlineStr">
@@ -39255,12 +39255,12 @@
       </c>
       <c r="BW64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY64" s="15" t="inlineStr">
@@ -39285,12 +39285,12 @@
       </c>
       <c r="CC64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE64" s="15" t="inlineStr">
@@ -39315,12 +39315,12 @@
       </c>
       <c r="CI64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CK64" s="15" t="inlineStr">
@@ -39345,12 +39345,12 @@
       </c>
       <c r="CO64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP64" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ64" s="15" t="inlineStr">
@@ -39800,17 +39800,17 @@
       </c>
       <c r="BK65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BL65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>s</t>
         </is>
       </c>
       <c r="BM65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BN65" s="15" t="inlineStr">
@@ -39825,17 +39825,17 @@
       </c>
       <c r="BP65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BQ65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BR65" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BS65" s="15" t="inlineStr">
@@ -39850,22 +39850,22 @@
       </c>
       <c r="BU65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BV65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BW65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="BX65" s="15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY65" s="15" t="inlineStr">
@@ -39875,42 +39875,42 @@
       </c>
       <c r="BZ65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CA65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>s</t>
         </is>
       </c>
       <c r="CB65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CC65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD65" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CF65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CG65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CH65" s="15" t="inlineStr">
@@ -39920,22 +39920,22 @@
       </c>
       <c r="CI65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CK65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CL65" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>|</t>
         </is>
       </c>
       <c r="CM65" s="15" t="inlineStr">
@@ -39950,12 +39950,12 @@
       </c>
       <c r="CO65" s="15" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CP65" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CQ65" s="15" t="inlineStr">
@@ -40410,22 +40410,22 @@
       </c>
       <c r="BL66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BM66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BN66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BO66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BP66" s="15" t="inlineStr">
@@ -40440,47 +40440,47 @@
       </c>
       <c r="BR66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BS66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BT66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BU66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BV66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BW66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BX66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BY66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="BZ66" s="15" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CA66" s="15" t="inlineStr">
@@ -40490,42 +40490,42 @@
       </c>
       <c r="CB66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CC66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CD66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CE66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CF66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CG66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CH66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CI66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CJ66" s="15" t="inlineStr">
@@ -40540,17 +40540,17 @@
       </c>
       <c r="CL66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CM66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CN66" s="15" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>~</t>
         </is>
       </c>
       <c r="CO66" s="15" t="inlineStr">
@@ -41050,12 +41050,12 @@
       </c>
       <c r="BS67" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>m</t>
         </is>
       </c>
       <c r="BT67" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BU67" s="15" t="inlineStr">
@@ -41100,12 +41100,12 @@
       </c>
       <c r="CC67" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>B</t>
         </is>
       </c>
       <c r="CD67" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CE67" s="15" t="inlineStr">
@@ -41655,12 +41655,12 @@
       </c>
       <c r="BS68" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BT68" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="BU68" s="15" t="inlineStr">
@@ -41705,12 +41705,12 @@
       </c>
       <c r="CC68" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CD68" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CE68" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Lab 11: Crypt lectern next to its gate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MSjWpMgByR7PswdtguveBk
</commit_message>
<xml_diff>
--- a/tools/world/lab11/lab11_layout.xlsx
+++ b/tools/world/lab11/lab11_layout.xlsx
@@ -31510,7 +31510,7 @@
       </c>
       <c r="CU51" s="15" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CV51" s="15" t="inlineStr">
@@ -57515,22 +57515,22 @@
       </c>
       <c r="CS94" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CT94" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="CU94" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CV94" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CW94" s="15" t="inlineStr">
@@ -58120,22 +58120,22 @@
       </c>
       <c r="CS95" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CT95" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CU95" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CV95" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CW95" s="15" t="inlineStr">
@@ -58725,22 +58725,22 @@
       </c>
       <c r="CS96" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CT96" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CU96" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>C</t>
         </is>
       </c>
       <c r="CV96" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>.</t>
         </is>
       </c>
       <c r="CW96" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Lab 11 Cistern: the tome is torn into four pages hidden in sunken chests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MSjWpMgByR7PswdtguveBk
</commit_message>
<xml_diff>
--- a/tools/world/lab11/lab11_layout.xlsx
+++ b/tools/world/lab11/lab11_layout.xlsx
@@ -94,7 +94,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="27">
+  <fills count="29">
     <fill>
       <patternFill/>
     </fill>
@@ -251,6 +251,18 @@
         <bgColor rgb="00503050"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D2B48C"/>
+        <bgColor rgb="00D2B48C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B7355"/>
+        <bgColor rgb="008B7355"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border/>
@@ -278,7 +290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -377,11 +389,17 @@
     <xf numFmtId="0" fontId="11" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="27">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -728,6 +746,32 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="00000000"/>
+        <sz val="8"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D2B48C"/>
+          <bgColor rgb="00D2B48C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="8"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="008B7355"/>
+          <bgColor rgb="008B7355"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <colors>
     <indexedColors>
@@ -45060,7 +45104,7 @@
       </c>
       <c r="Z74" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="AA74" s="15" t="inlineStr">
@@ -45315,7 +45359,7 @@
       </c>
       <c r="BY74" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="BZ74" s="15" t="inlineStr">
@@ -45385,7 +45429,7 @@
       </c>
       <c r="CM74" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="CN74" s="15" t="inlineStr">
@@ -52620,7 +52664,7 @@
       </c>
       <c r="CH86" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="CI86" s="15" t="inlineStr">
@@ -53080,7 +53124,7 @@
       </c>
       <c r="BE87" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="BF87" s="15" t="inlineStr">
@@ -57810,7 +57854,7 @@
       </c>
       <c r="AI95" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="AJ95" s="15" t="inlineStr">
@@ -57950,7 +57994,7 @@
       </c>
       <c r="BK95" s="15" t="inlineStr">
         <is>
-          <t>~</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="BL95" s="15" t="inlineStr">
@@ -62889,6 +62933,21 @@
     <cfRule type="expression" priority="38" dxfId="24" stopIfTrue="1">
       <formula>UPPER(B2)="SC"</formula>
     </cfRule>
+    <cfRule type="expression" priority="39" dxfId="25" stopIfTrue="1">
+      <formula>UPPER(B2)="P1"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="40" dxfId="25" stopIfTrue="1">
+      <formula>UPPER(B2)="P2"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="41" dxfId="25" stopIfTrue="1">
+      <formula>UPPER(B2)="P3"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="42" dxfId="25" stopIfTrue="1">
+      <formula>UPPER(B2)="P4"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="43" dxfId="26" stopIfTrue="1">
+      <formula>UPPER(B2)="CH"</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -62901,7 +62960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="32" min="1" max="1"/>
@@ -63433,13 +63492,74 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1" s="32"/>
-    <row r="51" ht="15.75" customHeight="1" s="32"/>
-    <row r="52" ht="15.75" customHeight="1" s="32"/>
-    <row r="53" ht="15.75" customHeight="1" s="32"/>
-    <row r="54" ht="15.75" customHeight="1" s="32"/>
+    <row r="50" ht="15.75" customHeight="1" s="32">
+      <c r="A50" s="38" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B50" s="34" t="inlineStr">
+        <is>
+          <t>sunken chest with torn page 1 (section 4 tome)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="32">
+      <c r="A51" s="38" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B51" s="34" t="inlineStr">
+        <is>
+          <t>sunken chest with torn page 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1" s="32">
+      <c r="A52" s="38" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B52" s="34" t="inlineStr">
+        <is>
+          <t>sunken chest with torn page 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="32">
+      <c r="A53" s="38" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B53" s="34" t="inlineStr">
+        <is>
+          <t>sunken chest with torn page 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1" s="32">
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="B54" s="34" t="inlineStr">
+        <is>
+          <t>sunken chest, only silt</t>
+        </is>
+      </c>
+    </row>
     <row r="55" ht="15.75" customHeight="1" s="32"/>
-    <row r="56" ht="15.75" customHeight="1" s="32"/>
+    <row r="56" ht="15.75" customHeight="1" s="32">
+      <c r="A56" s="34" t="inlineStr">
+        <is>
+          <t>Section 4's tome shelf (S4) only holds scraps: its tome is the four torn pages P1-P4, which players put together.</t>
+        </is>
+      </c>
+    </row>
     <row r="57" ht="15.75" customHeight="1" s="32"/>
     <row r="58" ht="15.75" customHeight="1" s="32"/>
     <row r="59" ht="15.75" customHeight="1" s="32"/>

</xml_diff>